<commit_message>
edit the manage student table and view report card and pagination
</commit_message>
<xml_diff>
--- a/Backend/abc.xlsx
+++ b/Backend/abc.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W2"/>
+  <dimension ref="A1:W12"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -541,9 +541,719 @@
         <v>Clear</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>d6660c84-58db-43c8-9b87-09c4187f8706</v>
+      </c>
+      <c r="B3" t="str">
+        <v>nikita sharma</v>
+      </c>
+      <c r="C3" t="str">
+        <v>raghuveer@gmail.com</v>
+      </c>
+      <c r="D3" t="str">
+        <v>7896541235</v>
+      </c>
+      <c r="E3" t="str">
+        <v>nikita@gmail.com</v>
+      </c>
+      <c r="F3" t="str">
+        <v xml:space="preserve">raghuveer </v>
+      </c>
+      <c r="G3" t="str">
+        <v>nirmala</v>
+      </c>
+      <c r="H3" t="str">
+        <v>7418529637</v>
+      </c>
+      <c r="I3" t="str">
+        <v>Female</v>
+      </c>
+      <c r="J3" t="str">
+        <v>asdfghjkl</v>
+      </c>
+      <c r="K3">
+        <v>123456</v>
+      </c>
+      <c r="L3" t="str">
+        <v>BBA+ITEG</v>
+      </c>
+      <c r="M3" t="str">
+        <v>2 Year</v>
+      </c>
+      <c r="N3" t="str">
+        <v>65</v>
+      </c>
+      <c r="O3">
+        <v>25</v>
+      </c>
+      <c r="P3" t="str">
+        <v>100</v>
+      </c>
+      <c r="Q3" t="str">
+        <v>65.00</v>
+      </c>
+      <c r="R3" t="str">
+        <v>Running</v>
+      </c>
+      <c r="S3" t="str">
+        <v>Running</v>
+      </c>
+      <c r="T3" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="U3" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="V3" t="str">
+        <v>Running</v>
+      </c>
+      <c r="W3" t="str">
+        <v>Running</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>2af63b9c-a7e2-4eb6-9f48-c630be0aa9f0</v>
+      </c>
+      <c r="B4" t="str">
+        <v>asdfghjkl</v>
+      </c>
+      <c r="C4" t="str">
+        <v>ghjk@gmail.com</v>
+      </c>
+      <c r="D4" t="str">
+        <v>7418526396</v>
+      </c>
+      <c r="E4" t="str">
+        <v>sdfghjk@gmial.com</v>
+      </c>
+      <c r="F4" t="str">
+        <v>sdfghjk</v>
+      </c>
+      <c r="G4" t="str">
+        <v>sdfghj</v>
+      </c>
+      <c r="H4" t="str">
+        <v>5678987654</v>
+      </c>
+      <c r="I4" t="str">
+        <v>Female</v>
+      </c>
+      <c r="J4" t="str">
+        <v>sdfghjk</v>
+      </c>
+      <c r="K4">
+        <v>1234560</v>
+      </c>
+      <c r="L4" t="str">
+        <v>DIPLOMA ITEG</v>
+      </c>
+      <c r="M4" t="str">
+        <v>3 Year</v>
+      </c>
+      <c r="N4" t="str">
+        <v>87</v>
+      </c>
+      <c r="O4">
+        <v>8</v>
+      </c>
+      <c r="P4" t="str">
+        <v>100</v>
+      </c>
+      <c r="Q4" t="str">
+        <v>87.00</v>
+      </c>
+      <c r="R4" t="str">
+        <v>Clear</v>
+      </c>
+      <c r="S4" t="str">
+        <v>Clear</v>
+      </c>
+      <c r="T4" t="str">
+        <v>Clear</v>
+      </c>
+      <c r="U4" t="str">
+        <v>Running</v>
+      </c>
+      <c r="V4" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="W4" t="str">
+        <v>Pending</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>a1f5d8f9-ce9d-4942-9a49-62cac84462b1</v>
+      </c>
+      <c r="B5" t="str">
+        <v>asdfghj</v>
+      </c>
+      <c r="C5" t="str">
+        <v>asdfghj@gmail.com</v>
+      </c>
+      <c r="D5" t="str">
+        <v>7418529632</v>
+      </c>
+      <c r="E5" t="str">
+        <v>asdf@gmail.com</v>
+      </c>
+      <c r="F5" t="str">
+        <v>uytreeri</v>
+      </c>
+      <c r="G5" t="str">
+        <v>sdfghj</v>
+      </c>
+      <c r="H5" t="str">
+        <v>7418529638</v>
+      </c>
+      <c r="I5" t="str">
+        <v>Female</v>
+      </c>
+      <c r="J5" t="str">
+        <v>sdfghj</v>
+      </c>
+      <c r="K5">
+        <v>12345</v>
+      </c>
+      <c r="L5" t="str">
+        <v>BBA+ITEG</v>
+      </c>
+      <c r="M5" t="str">
+        <v>3 Year</v>
+      </c>
+      <c r="N5" t="str">
+        <v>56</v>
+      </c>
+      <c r="O5">
+        <v>32</v>
+      </c>
+      <c r="P5" t="str">
+        <v>100</v>
+      </c>
+      <c r="Q5" t="str">
+        <v>56.00</v>
+      </c>
+      <c r="R5" t="str">
+        <v>Clear</v>
+      </c>
+      <c r="S5" t="str">
+        <v>Clear</v>
+      </c>
+      <c r="T5" t="str">
+        <v>Clear</v>
+      </c>
+      <c r="U5" t="str">
+        <v>Clear</v>
+      </c>
+      <c r="V5" t="str">
+        <v>Running</v>
+      </c>
+      <c r="W5" t="str">
+        <v>Pending</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>ef658948-a1f5-48f0-9082-e813a2688f59</v>
+      </c>
+      <c r="B6" t="str">
+        <v>nikita sharma</v>
+      </c>
+      <c r="C6" t="str">
+        <v>patient@gmail.com</v>
+      </c>
+      <c r="D6" t="str">
+        <v>7896541235</v>
+      </c>
+      <c r="E6" t="str">
+        <v>harshitayadav@gmail.com</v>
+      </c>
+      <c r="F6" t="str">
+        <v xml:space="preserve">raghuveer </v>
+      </c>
+      <c r="G6" t="str">
+        <v>nirmala</v>
+      </c>
+      <c r="H6" t="str">
+        <v>7418529637</v>
+      </c>
+      <c r="I6" t="str">
+        <v>Male</v>
+      </c>
+      <c r="J6" t="str">
+        <v>asdfghjkl</v>
+      </c>
+      <c r="K6">
+        <v>123</v>
+      </c>
+      <c r="L6" t="str">
+        <v>DIPLOMA ITEG</v>
+      </c>
+      <c r="M6" t="str">
+        <v>2 Year</v>
+      </c>
+      <c r="N6" t="str">
+        <v>85</v>
+      </c>
+      <c r="O6">
+        <v>12</v>
+      </c>
+      <c r="P6" t="str">
+        <v>100</v>
+      </c>
+      <c r="Q6" t="str">
+        <v>85.00</v>
+      </c>
+      <c r="R6" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="S6" t="str">
+        <v>Clear</v>
+      </c>
+      <c r="T6" t="str">
+        <v>Running</v>
+      </c>
+      <c r="U6" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="V6" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="W6" t="str">
+        <v>Running</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>80eb160c-722b-4c60-8f37-4ad28ff65e16</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Harshita yadav</v>
+      </c>
+      <c r="C7" t="str">
+        <v>dfghj@gmail.com</v>
+      </c>
+      <c r="D7" t="str">
+        <v>7896541256</v>
+      </c>
+      <c r="E7" t="str">
+        <v>haeshi@gmail.com</v>
+      </c>
+      <c r="F7" t="str">
+        <v>sdfghjk</v>
+      </c>
+      <c r="G7" t="str">
+        <v>nirmala</v>
+      </c>
+      <c r="H7" t="str">
+        <v>7418529637</v>
+      </c>
+      <c r="I7" t="str">
+        <v>Female</v>
+      </c>
+      <c r="J7" t="str">
+        <v>jhgfsdf</v>
+      </c>
+      <c r="K7">
+        <v>123</v>
+      </c>
+      <c r="L7" t="str">
+        <v>BCA+ITEG</v>
+      </c>
+      <c r="M7" t="str">
+        <v>2 Year</v>
+      </c>
+      <c r="N7" t="str">
+        <v>85</v>
+      </c>
+      <c r="O7">
+        <v>4</v>
+      </c>
+      <c r="P7" t="str">
+        <v>100</v>
+      </c>
+      <c r="Q7" t="str">
+        <v>85.00</v>
+      </c>
+      <c r="R7" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="S7" t="str">
+        <v>Running</v>
+      </c>
+      <c r="T7" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="U7" t="str">
+        <v>Running</v>
+      </c>
+      <c r="V7" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="W7" t="str">
+        <v>Pending</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>8d96b2dc-e519-46dd-bab5-17a74d862977</v>
+      </c>
+      <c r="B8" t="str">
+        <v>sdfgfdsdf</v>
+      </c>
+      <c r="C8" t="str">
+        <v>dfghj@gmial.com</v>
+      </c>
+      <c r="D8" t="str">
+        <v>5678976546</v>
+      </c>
+      <c r="E8" t="str">
+        <v>asdfg@gmial.com</v>
+      </c>
+      <c r="F8" t="str">
+        <v>gfdsdfs</v>
+      </c>
+      <c r="G8" t="str">
+        <v>hgfdsfgb</v>
+      </c>
+      <c r="H8" t="str">
+        <v>9876543234</v>
+      </c>
+      <c r="I8" t="str">
+        <v>Female</v>
+      </c>
+      <c r="J8" t="str">
+        <v>lkjhgffghj</v>
+      </c>
+      <c r="K8">
+        <v>412</v>
+      </c>
+      <c r="L8" t="str">
+        <v>DIPLOMA ITEG</v>
+      </c>
+      <c r="M8" t="str">
+        <v>1 Year</v>
+      </c>
+      <c r="N8" t="str">
+        <v>76</v>
+      </c>
+      <c r="O8">
+        <v>20</v>
+      </c>
+      <c r="P8" t="str">
+        <v>100</v>
+      </c>
+      <c r="Q8" t="str">
+        <v>76.00</v>
+      </c>
+      <c r="R8" t="str">
+        <v>Running</v>
+      </c>
+      <c r="S8" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="T8" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="U8" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="V8" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="W8" t="str">
+        <v>Pending</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>52dec3a7-cdc6-4424-9bc6-ea5aa01d9376</v>
+      </c>
+      <c r="B9" t="str">
+        <v>sdfghjk</v>
+      </c>
+      <c r="C9" t="str">
+        <v>sdfghj@gmail.com</v>
+      </c>
+      <c r="D9" t="str">
+        <v>7896541235</v>
+      </c>
+      <c r="E9" t="str">
+        <v>sdfgh@gmail.com</v>
+      </c>
+      <c r="F9" t="str">
+        <v>sdfghj</v>
+      </c>
+      <c r="G9" t="str">
+        <v>meena</v>
+      </c>
+      <c r="H9" t="str">
+        <v>7418529632</v>
+      </c>
+      <c r="I9" t="str">
+        <v>Male</v>
+      </c>
+      <c r="J9" t="str">
+        <v>asdfghjkgf</v>
+      </c>
+      <c r="K9">
+        <v>23</v>
+      </c>
+      <c r="L9" t="str">
+        <v>BCA+ITEG</v>
+      </c>
+      <c r="M9" t="str">
+        <v>3 Year</v>
+      </c>
+      <c r="N9" t="str">
+        <v>46</v>
+      </c>
+      <c r="O9">
+        <v>54</v>
+      </c>
+      <c r="P9" t="str">
+        <v>100</v>
+      </c>
+      <c r="Q9" t="str">
+        <v>46.00</v>
+      </c>
+      <c r="R9" t="str">
+        <v>Clear</v>
+      </c>
+      <c r="S9" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="T9" t="str">
+        <v>Running</v>
+      </c>
+      <c r="U9" t="str">
+        <v>Running</v>
+      </c>
+      <c r="V9" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="W9" t="str">
+        <v>Pending</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>0f055919-ea6d-46fb-978a-470863c7f4ab</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Surbhi rajput</v>
+      </c>
+      <c r="C10" t="str">
+        <v>sdfghgfd@gmail.com</v>
+      </c>
+      <c r="D10" t="str">
+        <v>7418523698</v>
+      </c>
+      <c r="E10" t="str">
+        <v>surbhi@gmail.com</v>
+      </c>
+      <c r="F10" t="str">
+        <v xml:space="preserve">raghuveer </v>
+      </c>
+      <c r="G10" t="str">
+        <v>nirmala</v>
+      </c>
+      <c r="H10" t="str">
+        <v>7987777821</v>
+      </c>
+      <c r="I10" t="str">
+        <v>Female</v>
+      </c>
+      <c r="J10" t="str">
+        <v>asdfghjk</v>
+      </c>
+      <c r="K10">
+        <v>741852</v>
+      </c>
+      <c r="L10" t="str">
+        <v>BBA+ITEG</v>
+      </c>
+      <c r="M10" t="str">
+        <v>3 Year</v>
+      </c>
+      <c r="N10" t="str">
+        <v>85</v>
+      </c>
+      <c r="O10">
+        <v>25</v>
+      </c>
+      <c r="P10" t="str">
+        <v>100</v>
+      </c>
+      <c r="Q10" t="str">
+        <v>85.00</v>
+      </c>
+      <c r="R10" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="S10" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="T10" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="U10" t="str">
+        <v>Running</v>
+      </c>
+      <c r="V10" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="W10" t="str">
+        <v>Pending</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>f99d4ec1-c0b8-4030-93e6-dfe8407efc98</v>
+      </c>
+      <c r="B11" t="str">
+        <v>kjhgfd</v>
+      </c>
+      <c r="C11" t="str">
+        <v>sdfgh@gmail.com</v>
+      </c>
+      <c r="D11" t="str">
+        <v>7418529632</v>
+      </c>
+      <c r="E11" t="str">
+        <v>iuyty@gmail.com</v>
+      </c>
+      <c r="F11" t="str">
+        <v>kjhgfd</v>
+      </c>
+      <c r="G11" t="str">
+        <v>fghjkl</v>
+      </c>
+      <c r="H11" t="str">
+        <v>7418529632</v>
+      </c>
+      <c r="I11" t="str">
+        <v>Male</v>
+      </c>
+      <c r="J11" t="str">
+        <v>wertyuoiuy</v>
+      </c>
+      <c r="K11">
+        <v>7418529632</v>
+      </c>
+      <c r="L11" t="str">
+        <v>BBA+ITEG</v>
+      </c>
+      <c r="M11" t="str">
+        <v>1 Year</v>
+      </c>
+      <c r="N11" t="str">
+        <v>45</v>
+      </c>
+      <c r="O11">
+        <v>52</v>
+      </c>
+      <c r="P11" t="str">
+        <v>99</v>
+      </c>
+      <c r="Q11" t="str">
+        <v>45.45</v>
+      </c>
+      <c r="R11" t="str">
+        <v>Running</v>
+      </c>
+      <c r="S11" t="str">
+        <v>Clear</v>
+      </c>
+      <c r="T11" t="str">
+        <v>Running</v>
+      </c>
+      <c r="U11" t="str">
+        <v>Running</v>
+      </c>
+      <c r="V11" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="W11" t="str">
+        <v>Pending</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>f10c9081-d035-4f42-8f53-3112d7d49119</v>
+      </c>
+      <c r="B12" t="str">
+        <v>sonu vyas</v>
+      </c>
+      <c r="C12" t="str">
+        <v>ram@gmail.com</v>
+      </c>
+      <c r="D12" t="str">
+        <v>7418523698</v>
+      </c>
+      <c r="E12" t="str">
+        <v>sonu990@gmail.com</v>
+      </c>
+      <c r="F12" t="str">
+        <v>ram</v>
+      </c>
+      <c r="G12" t="str">
+        <v>reena</v>
+      </c>
+      <c r="H12" t="str">
+        <v>1236547898</v>
+      </c>
+      <c r="I12" t="str">
+        <v>Female</v>
+      </c>
+      <c r="J12" t="str">
+        <v>olmkjuygg</v>
+      </c>
+      <c r="K12">
+        <v>741852963</v>
+      </c>
+      <c r="L12" t="str">
+        <v>BBA+ITEG</v>
+      </c>
+      <c r="M12" t="str">
+        <v>4 Year</v>
+      </c>
+      <c r="N12" t="str">
+        <v>74</v>
+      </c>
+      <c r="O12">
+        <v>12</v>
+      </c>
+      <c r="P12" t="str">
+        <v>100</v>
+      </c>
+      <c r="Q12" t="str">
+        <v>74.00</v>
+      </c>
+      <c r="R12" t="str">
+        <v>Running</v>
+      </c>
+      <c r="S12" t="str">
+        <v>Running</v>
+      </c>
+      <c r="T12" t="str">
+        <v>Clear</v>
+      </c>
+      <c r="U12" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="V12" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="W12" t="str">
+        <v>Pending</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W12"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update - sidebar , teacher home, student table, generate report card
</commit_message>
<xml_diff>
--- a/Backend/abc.xlsx
+++ b/Backend/abc.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W12"/>
+  <dimension ref="A1:W13"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1251,9 +1251,80 @@
         <v>Pending</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>d02ad3ba-1248-4321-84f7-42da31c79096</v>
+      </c>
+      <c r="B13" t="str">
+        <v>asdfgh</v>
+      </c>
+      <c r="C13" t="str">
+        <v>dfgh@gmail.com</v>
+      </c>
+      <c r="D13" t="str">
+        <v>9987654322</v>
+      </c>
+      <c r="E13" t="str">
+        <v>dfgh@gmial.com</v>
+      </c>
+      <c r="F13" t="str">
+        <v>sdfgh</v>
+      </c>
+      <c r="G13" t="str">
+        <v>dfghj</v>
+      </c>
+      <c r="H13" t="str">
+        <v>1234567876</v>
+      </c>
+      <c r="I13" t="str">
+        <v>Female</v>
+      </c>
+      <c r="J13" t="str">
+        <v>asdfghj</v>
+      </c>
+      <c r="K13">
+        <v>123456</v>
+      </c>
+      <c r="L13" t="str">
+        <v>BCA+ITEG</v>
+      </c>
+      <c r="M13" t="str">
+        <v>2 Year</v>
+      </c>
+      <c r="N13" t="str">
+        <v>12</v>
+      </c>
+      <c r="O13">
+        <v>76</v>
+      </c>
+      <c r="P13" t="str">
+        <v>100</v>
+      </c>
+      <c r="Q13" t="str">
+        <v>12.00</v>
+      </c>
+      <c r="R13" t="str">
+        <v>Clear</v>
+      </c>
+      <c r="S13" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="T13" t="str">
+        <v>Running</v>
+      </c>
+      <c r="U13" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="V13" t="str">
+        <v>Running</v>
+      </c>
+      <c r="W13" t="str">
+        <v>Running</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>